<commit_message>
[IMP] Disposal on close asset
</commit_message>
<xml_diff>
--- a/assets_management/tests/data/account_invoice.xlsx
+++ b/assets_management/tests/data/account_invoice.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -91,16 +91,28 @@
     <t xml:space="preserve">external.INV</t>
   </si>
   <si>
-    <t xml:space="preserve">z0bug.sale_invoice_1</t>
+    <t xml:space="preserve">z0bug.sale_invoice_2</t>
   </si>
   <si>
     <t xml:space="preserve">base.res_partner_18</t>
   </si>
   <si>
-    <t xml:space="preserve">Asset #1 and #2</t>
+    <t xml:space="preserve">Asset #2</t>
   </si>
   <si>
     <t xml:space="preserve">####-01-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">z0bug.sale_invoice_13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">base.res_partner_10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset #1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">####-01-15</t>
   </si>
 </sst>
 </file>
@@ -334,7 +346,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.97"/>
@@ -454,6 +466,27 @@
         <v>22</v>
       </c>
     </row>
+    <row r="6" s="4" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>